<commit_message>
added delete customer test script
</commit_message>
<xml_diff>
--- a/data/TestScriptData.xlsx
+++ b/data/TestScriptData.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rathan Kumar S M\eclipse-workspace\Selenium-Automation\Actitime\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4533B708-E293-42F3-993C-4168FB619AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7FFE16-38BD-4867-9D4D-DC0E37A84D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="2" xr2:uid="{A104AA2B-88B9-41DB-B737-F45ECBC5C67B}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="19">
   <si>
     <t>Test-ID</t>
   </si>
@@ -81,12 +81,16 @@
   </si>
   <si>
     <t>pass</t>
+  </si>
+  <si>
+    <t>modified KOTAK_5091</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -455,49 +459,49 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="14.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.26953125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="13.7265625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="18.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
@@ -511,56 +515,56 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="6.6328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="14.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.26953125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="17.36328125"/>
+    <col min="5" max="6" bestFit="true" customWidth="true" width="18.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" t="s" s="0">
         <v>15</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" t="s" s="0">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" t="s" s="0">
         <v>17</v>
       </c>
     </row>
@@ -574,45 +578,45 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="6.6328125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="14.81640625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="15.26953125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="18.54296875"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="18.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
+      <c r="D2" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>